<commit_message>
T-0065: link 97 Supreme Court cases and statutes to Oyez, the Library of Congress and govinfo
Matrix links 39 -> 136 of 384. editorial/backfill_links.py proposes each link from
its citation and checks it (Oyez's own citation data; govinfo PDF header names the
public law) before writing; blanks only. Report in editorial/object-links-report.json.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Object_Matrix.xlsx
+++ b/editorial/NTK_Backstory_Object_Matrix.xlsx
@@ -4020,7 +4020,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O51" s="2" t="n"/>
+      <c r="O51" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1789-1850/5us137</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
@@ -6084,7 +6088,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O81" s="2" t="n"/>
+      <c r="O81" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1789-1850/36us420</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
@@ -6151,7 +6159,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O82" s="2" t="n"/>
+      <c r="O82" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1789-1850/36us420</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
@@ -7046,7 +7058,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O95" s="2" t="n"/>
+      <c r="O95" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/60us393</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="n">
@@ -8580,7 +8596,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O117" s="2" t="n"/>
+      <c r="O117" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/83us36</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="n">
@@ -8793,7 +8813,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O120" s="2" t="n"/>
+      <c r="O120" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/94us113</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="n">
@@ -8864,7 +8888,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O121" s="2" t="n"/>
+      <c r="O121" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/94us113</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="n">
@@ -9057,7 +9085,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O124" s="2" t="n"/>
+      <c r="O124" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/22/58</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="n">
@@ -9128,7 +9160,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O125" s="2" t="n"/>
+      <c r="O125" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/109us3</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="n">
@@ -9199,7 +9235,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O126" s="2" t="n"/>
+      <c r="O126" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/109us3</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="n">
@@ -10157,7 +10197,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O140" s="2" t="n"/>
+      <c r="O140" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/156us1</t>
+        </is>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="n">
@@ -10228,7 +10272,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O141" s="2" t="n"/>
+      <c r="O141" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/156us1</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="n">
@@ -10299,7 +10347,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O142" s="2" t="n"/>
+      <c r="O142" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/157us429</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" s="2" t="n">
@@ -10370,7 +10422,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O143" s="2" t="n"/>
+      <c r="O143" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/157us429</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="n">
@@ -10508,7 +10564,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O145" s="2" t="n"/>
+      <c r="O145" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/163us537</t>
+        </is>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="n">
@@ -10579,7 +10639,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O146" s="2" t="n"/>
+      <c r="O146" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1850-1900/163us537</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="n">
@@ -11269,7 +11333,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O156" s="2" t="n"/>
+      <c r="O156" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/198us45</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="n">
@@ -11340,7 +11408,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O157" s="2" t="n"/>
+      <c r="O157" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/198us45</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="n">
@@ -11549,7 +11621,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O160" s="2" t="n"/>
+      <c r="O160" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/208us412</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="n">
@@ -12223,7 +12299,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O170" s="2" t="n"/>
+      <c r="O170" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/39/675</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="n">
@@ -12574,7 +12654,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O175" s="2" t="n"/>
+      <c r="O175" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/247us251</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="n">
@@ -12645,7 +12729,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O176" s="2" t="n"/>
+      <c r="O176" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/247us251</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="n">
@@ -12779,7 +12867,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O178" s="2" t="n"/>
+      <c r="O178" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/41/305</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="n">
@@ -12846,7 +12938,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O179" s="2" t="n"/>
+      <c r="O179" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/250us616</t>
+        </is>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="n">
@@ -12917,7 +13013,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O180" s="2" t="n"/>
+      <c r="O180" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/250us616</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" s="2" t="n">
@@ -13185,7 +13285,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O184" s="2" t="n"/>
+      <c r="O184" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/43/153</t>
+        </is>
+      </c>
     </row>
     <row r="185">
       <c r="A185" s="2" t="n">
@@ -13386,7 +13490,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O187" s="2" t="n"/>
+      <c r="O187" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/283us697</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="n">
@@ -13591,7 +13699,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O190" s="2" t="n"/>
+      <c r="O190" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/49/620</t>
+        </is>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="n">
@@ -13662,7 +13774,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O191" s="2" t="n"/>
+      <c r="O191" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/297us1</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="n">
@@ -13733,7 +13849,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O192" s="2" t="n"/>
+      <c r="O192" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1900-1940/297us1</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="n">
@@ -15531,7 +15651,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O218" s="2" t="n"/>
+      <c r="O218" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1940-1955/347us483</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="n">
@@ -15665,7 +15789,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O220" s="2" t="n"/>
+      <c r="O220" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/69/7</t>
+        </is>
+      </c>
     </row>
     <row r="221">
       <c r="A221" s="2" t="n">
@@ -16008,7 +16136,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O225" s="2" t="n"/>
+      <c r="O225" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1960/236</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" s="2" t="n">
@@ -16142,7 +16274,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O227" s="2" t="n"/>
+      <c r="O227" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1961/468</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" s="2" t="n">
@@ -16339,7 +16475,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O230" s="2" t="n"/>
+      <c r="O230" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1963/39</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" s="2" t="n">
@@ -16402,7 +16542,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O231" s="2" t="n"/>
+      <c r="O231" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1962/155</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" s="2" t="n">
@@ -16465,7 +16609,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O232" s="2" t="n"/>
+      <c r="O232" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1962/142</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" s="2" t="n">
@@ -16808,7 +16956,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O237" s="2" t="n"/>
+      <c r="O237" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1963/23</t>
+        </is>
+      </c>
     </row>
     <row r="238">
       <c r="A238" s="2" t="n">
@@ -16879,7 +17031,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O238" s="2" t="n"/>
+      <c r="O238" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1963/23</t>
+        </is>
+      </c>
     </row>
     <row r="239">
       <c r="A239" s="2" t="n">
@@ -17356,7 +17512,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O245" s="2" t="n"/>
+      <c r="O245" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1965/759</t>
+        </is>
+      </c>
     </row>
     <row r="246">
       <c r="A246" s="2" t="n">
@@ -17490,7 +17650,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O247" s="2" t="n"/>
+      <c r="O247" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/82/197</t>
+        </is>
+      </c>
     </row>
     <row r="248">
       <c r="A248" s="2" t="n">
@@ -17616,7 +17780,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O249" s="2" t="n"/>
+      <c r="O249" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/82/1213</t>
+        </is>
+      </c>
     </row>
     <row r="250">
       <c r="A250" s="2" t="n">
@@ -17888,7 +18056,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O253" s="2" t="n"/>
+      <c r="O253" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1968/2</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="2" t="n">
@@ -18424,7 +18596,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O261" s="2" t="n"/>
+      <c r="O261" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/84/1676</t>
+        </is>
+      </c>
     </row>
     <row r="262">
       <c r="A262" s="4" t="n">
@@ -18487,7 +18663,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O262" s="2" t="n"/>
+      <c r="O262" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1970/1873</t>
+        </is>
+      </c>
     </row>
     <row r="263">
       <c r="A263" s="4" t="n">
@@ -18952,7 +19132,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O269" s="2" t="n"/>
+      <c r="O269" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1971/70-110</t>
+        </is>
+      </c>
     </row>
     <row r="270">
       <c r="A270" s="4" t="n">
@@ -19555,7 +19739,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O278" s="2" t="n"/>
+      <c r="O278" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1979/76-811</t>
+        </is>
+      </c>
     </row>
     <row r="279">
       <c r="A279" s="4" t="n">
@@ -19689,7 +19877,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O280" s="2" t="n"/>
+      <c r="O280" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/93/14</t>
+        </is>
+      </c>
     </row>
     <row r="281">
       <c r="A281" s="4" t="n">
@@ -19961,7 +20153,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O284" s="2" t="n"/>
+      <c r="O284" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1979/78-1007</t>
+        </is>
+      </c>
     </row>
     <row r="285">
       <c r="A285" s="4" t="n">
@@ -20032,7 +20228,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O285" s="2" t="n"/>
+      <c r="O285" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1979/78-1007</t>
+        </is>
+      </c>
     </row>
     <row r="286">
       <c r="A286" s="4" t="n">
@@ -20485,7 +20685,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O292" s="2" t="n"/>
+      <c r="O292" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1981/80-1538</t>
+        </is>
+      </c>
     </row>
     <row r="293">
       <c r="A293" s="4" t="n">
@@ -20737,7 +20941,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O296" s="2" t="n"/>
+      <c r="O296" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1983/82-1005</t>
+        </is>
+      </c>
     </row>
     <row r="297">
       <c r="A297" s="4" t="n">
@@ -20800,7 +21008,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O297" s="2" t="n"/>
+      <c r="O297" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1985/85-140</t>
+        </is>
+      </c>
     </row>
     <row r="298">
       <c r="A298" s="4" t="n">
@@ -21237,7 +21449,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O304" s="2" t="n"/>
+      <c r="O304" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1989/88-1213</t>
+        </is>
+      </c>
     </row>
     <row r="305">
       <c r="A305" s="4" t="n">
@@ -21493,7 +21709,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O308" s="2" t="n"/>
+      <c r="O308" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/105/1071</t>
+        </is>
+      </c>
     </row>
     <row r="309">
       <c r="A309" s="4" t="n">
@@ -21556,7 +21776,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O309" s="2" t="n"/>
+      <c r="O309" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1991/91-744</t>
+        </is>
+      </c>
     </row>
     <row r="310">
       <c r="A310" s="4" t="n">
@@ -21619,7 +21843,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O310" s="2" t="n"/>
+      <c r="O310" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/107/6</t>
+        </is>
+      </c>
     </row>
     <row r="311">
       <c r="A311" s="4" t="n">
@@ -21682,7 +21910,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O311" s="2" t="n"/>
+      <c r="O311" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/107/1488</t>
+        </is>
+      </c>
     </row>
     <row r="312">
       <c r="A312" s="4" t="n">
@@ -21808,7 +22040,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O313" s="2" t="n"/>
+      <c r="O313" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/statute/108/1796</t>
+        </is>
+      </c>
     </row>
     <row r="314">
       <c r="A314" s="4" t="n">
@@ -22127,7 +22363,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O318" s="2" t="n"/>
+      <c r="O318" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/104/public/104?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="319">
       <c r="A319" s="4" t="n">
@@ -22190,7 +22430,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O319" s="2" t="n"/>
+      <c r="O319" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/104/public/193?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="320">
       <c r="A320" s="4" t="n">
@@ -22253,7 +22497,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O320" s="2" t="n"/>
+      <c r="O320" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/104/public/199?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="321">
       <c r="A321" s="4" t="n">
@@ -22316,7 +22564,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O321" s="2" t="n"/>
+      <c r="O321" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/104/public/208?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="322">
       <c r="A322" s="4" t="n">
@@ -22379,7 +22631,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O322" s="2" t="n"/>
+      <c r="O322" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1996/96-511</t>
+        </is>
+      </c>
     </row>
     <row r="323">
       <c r="A323" s="4" t="n">
@@ -22442,7 +22698,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O323" s="2" t="n"/>
+      <c r="O323" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/106/public/102?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="324">
       <c r="A324" s="4" t="n">
@@ -22505,7 +22765,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O324" s="2" t="n"/>
+      <c r="O324" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/1999/99-138</t>
+        </is>
+      </c>
     </row>
     <row r="325">
       <c r="A325" s="4" t="n">
@@ -22631,7 +22895,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O326" s="2" t="n"/>
+      <c r="O326" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2000/00-949</t>
+        </is>
+      </c>
     </row>
     <row r="327">
       <c r="A327" s="4" t="n">
@@ -22694,7 +22962,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O327" s="2" t="n"/>
+      <c r="O327" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/107/public/40?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="328">
       <c r="A328" s="4" t="n">
@@ -22820,7 +23092,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O329" s="2" t="n"/>
+      <c r="O329" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/107/public/56?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="330">
       <c r="A330" s="4" t="n">
@@ -22883,7 +23159,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O330" s="2" t="n"/>
+      <c r="O330" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/107/public/110?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="331">
       <c r="A331" s="4" t="n">
@@ -23072,7 +23352,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O333" s="2" t="n"/>
+      <c r="O333" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/107/public/243?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="334">
       <c r="A334" s="4" t="n">
@@ -23198,7 +23482,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O335" s="2" t="n"/>
+      <c r="O335" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2002/02-241</t>
+        </is>
+      </c>
     </row>
     <row r="336">
       <c r="A336" s="4" t="n">
@@ -23261,7 +23549,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O336" s="2" t="n"/>
+      <c r="O336" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2002/02-102</t>
+        </is>
+      </c>
     </row>
     <row r="337">
       <c r="A337" s="4" t="n">
@@ -23576,7 +23868,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O341" s="2" t="n"/>
+      <c r="O341" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2006/05-1120</t>
+        </is>
+      </c>
     </row>
     <row r="342">
       <c r="A342" s="4" t="n">
@@ -23706,7 +24002,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O343" s="2" t="n"/>
+      <c r="O343" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2007/07-290</t>
+        </is>
+      </c>
     </row>
     <row r="344">
       <c r="A344" s="4" t="n">
@@ -23769,7 +24069,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O344" s="2" t="n"/>
+      <c r="O344" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/110/public/343?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="345">
       <c r="A345" s="4" t="n">
@@ -23962,7 +24266,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O347" s="2" t="n"/>
+      <c r="O347" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2008/08-205</t>
+        </is>
+      </c>
     </row>
     <row r="348">
       <c r="A348" s="2" t="n">
@@ -24025,7 +24333,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O348" s="2" t="n"/>
+      <c r="O348" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/111/public/148?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="349">
       <c r="A349" s="2" t="n">
@@ -24151,7 +24463,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O350" s="2" t="n"/>
+      <c r="O350" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2009/08-1521</t>
+        </is>
+      </c>
     </row>
     <row r="351">
       <c r="A351" s="2" t="n">
@@ -24214,7 +24530,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O351" s="2" t="n"/>
+      <c r="O351" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/111/public/203?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="352">
       <c r="A352" s="2" t="n">
@@ -24403,7 +24723,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O354" s="2" t="n"/>
+      <c r="O354" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2011/11-182</t>
+        </is>
+      </c>
     </row>
     <row r="355">
       <c r="A355" s="2" t="n">
@@ -24466,7 +24790,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O355" s="2" t="n"/>
+      <c r="O355" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2011/11-393</t>
+        </is>
+      </c>
     </row>
     <row r="356">
       <c r="A356" s="2" t="n">
@@ -24529,7 +24857,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O356" s="2" t="n"/>
+      <c r="O356" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2012/12-96</t>
+        </is>
+      </c>
     </row>
     <row r="357">
       <c r="A357" s="2" t="n">
@@ -24592,7 +24924,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O357" s="2" t="n"/>
+      <c r="O357" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2012/12-307</t>
+        </is>
+      </c>
     </row>
     <row r="358">
       <c r="A358" s="2" t="n">
@@ -24722,7 +25058,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O359" s="2" t="n"/>
+      <c r="O359" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2013/13-354</t>
+        </is>
+      </c>
     </row>
     <row r="360">
       <c r="A360" s="2" t="n">
@@ -24785,7 +25125,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O360" s="2" t="n"/>
+      <c r="O360" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2014/14-556</t>
+        </is>
+      </c>
     </row>
     <row r="361">
       <c r="A361" s="2" t="n">
@@ -25293,7 +25637,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O368" s="2" t="n"/>
+      <c r="O368" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/115/public/97?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="369">
       <c r="A369" s="2" t="n">
@@ -25419,7 +25767,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O370" s="2" t="n"/>
+      <c r="O370" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2017/16-111</t>
+        </is>
+      </c>
     </row>
     <row r="371">
       <c r="A371" s="2" t="n">
@@ -25545,7 +25897,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O372" s="2" t="n"/>
+      <c r="O372" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2018/18-422</t>
+        </is>
+      </c>
     </row>
     <row r="373">
       <c r="A373" s="2" t="n">
@@ -25734,7 +26090,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O375" s="2" t="n"/>
+      <c r="O375" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2019/17-1618</t>
+        </is>
+      </c>
     </row>
     <row r="376">
       <c r="A376" s="2" t="n">
@@ -25860,7 +26220,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O377" s="2" t="n"/>
+      <c r="O377" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2021/20-843</t>
+        </is>
+      </c>
     </row>
     <row r="378">
       <c r="A378" s="2" t="n">
@@ -25923,7 +26287,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O378" s="2" t="n"/>
+      <c r="O378" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2021/19-1392</t>
+        </is>
+      </c>
     </row>
     <row r="379">
       <c r="A379" s="2" t="n">
@@ -25986,7 +26354,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O379" s="2" t="n"/>
+      <c r="O379" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2021/20-1530</t>
+        </is>
+      </c>
     </row>
     <row r="380">
       <c r="A380" s="2" t="n">
@@ -26049,7 +26421,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O380" s="2" t="n"/>
+      <c r="O380" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/link/plaw/117/public/169?link-type=pdf</t>
+        </is>
+      </c>
     </row>
     <row r="381">
       <c r="A381" s="2" t="n">
@@ -26175,7 +26551,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O382" s="2" t="n"/>
+      <c r="O382" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2022/20-1199</t>
+        </is>
+      </c>
     </row>
     <row r="383">
       <c r="A383" s="2" t="n">
@@ -26238,7 +26618,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O383" s="2" t="n"/>
+      <c r="O383" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2023/22-451</t>
+        </is>
+      </c>
     </row>
     <row r="384">
       <c r="A384" s="2" t="n">
@@ -26301,7 +26685,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O384" s="2" t="n"/>
+      <c r="O384" s="2" t="inlineStr">
+        <is>
+          <t>https://www.oyez.org/cases/2023/23-939</t>
+        </is>
+      </c>
     </row>
     <row r="385">
       <c r="A385" s="2" t="n">

</xml_diff>

<commit_message>
T-0065: link 118 more objects to primary sources (Hofstadter items, Presidential papers, other)
Found by seven parallel research passes, each link re-fetched and content-checked
independently before writing. Verified links only; 45 probable and 78 not found held back.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Object_Matrix.xlsx
+++ b/editorial/NTK_Backstory_Object_Matrix.xlsx
@@ -625,7 +625,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O2" s="2" t="n"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ruhr-uni-bochum.de/gna/Quellensammlung/01/01_govenorglenroleofindians_1761.htm</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="n">
@@ -972,7 +976,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O7" s="2" t="n"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/resolu65.asp</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
@@ -1390,7 +1398,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O13" s="2" t="n"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/resolves.asp</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
@@ -1674,7 +1686,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O17" s="2" t="n"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/arms.asp</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
@@ -1808,7 +1824,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O19" s="2" t="n"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/bim_eighteenth-century_deceiver-unmasked-the_inglis-charles-bishop-_1776</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="n">
@@ -1879,7 +1899,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O20" s="2" t="n"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/files/147/147-h/147-h.htm</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="n">
@@ -1950,7 +1974,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O21" s="2" t="n"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>https://www.econlib.org/library/Smith/smWN.html?chapter_num=32#book-reader</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="n">
@@ -2021,7 +2049,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O22" s="2" t="n"/>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>https://www.econlib.org/library/Smith/smWN.html?chapter_num=33#book-reader</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
@@ -2226,7 +2258,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O25" s="2" t="n"/>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>https://www.archives.gov/founding-docs/declaration-transcript</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
@@ -2360,7 +2396,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O27" s="2" t="n"/>
+      <c r="O27" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/notes-on-the-state-of-virginia-2/</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="n">
@@ -2632,7 +2672,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O31" s="2" t="n"/>
+      <c r="O31" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/debates_609.asp</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
@@ -2695,7 +2739,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O32" s="2" t="n"/>
+      <c r="O32" s="2" t="inlineStr">
+        <is>
+          <t>https://www.archives.gov/founding-docs/constitution-transcript</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
@@ -2766,7 +2814,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O33" s="2" t="n"/>
+      <c r="O33" s="2" t="inlineStr">
+        <is>
+          <t>https://www.consource.org/document/elbridge-gerry-to-president-of-senate-and-speaker-of-house-of-representatives-of-massachusetts-1787-10-18/</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
@@ -3255,7 +3307,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O40" s="2" t="n"/>
+      <c r="O40" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/bank-tj.asp</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
@@ -3326,7 +3382,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O41" s="2" t="n"/>
+      <c r="O41" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/bank-ah.asp</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
@@ -3669,7 +3729,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O46" s="2" t="n"/>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/washing.asp</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
@@ -3878,7 +3942,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O49" s="2" t="n"/>
+      <c r="O49" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/19th_century/jefinau1.asp</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
@@ -4369,7 +4437,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O56" s="2" t="n"/>
+      <c r="O56" s="2" t="inlineStr">
+        <is>
+          <t>https://millercenter.org/the-presidency/presidential-speeches/june-1-1812-special-message-congress-foreign-policy-crisis-war</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
@@ -4578,7 +4650,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O59" s="2" t="n"/>
+      <c r="O59" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/letter-to-judge-spencer-roane/</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
@@ -4716,7 +4792,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O61" s="2" t="n"/>
+      <c r="O61" s="2" t="inlineStr">
+        <is>
+          <t>https://www.primarysourcecoop.org/publications/jqa/document/jqadiaries-v34-1823-11-p149--entry1?redirectFromPubs=1</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
@@ -4787,7 +4867,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O62" s="2" t="n"/>
+      <c r="O62" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/19th_century/monroe.asp</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
@@ -4858,7 +4942,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O63" s="2" t="n"/>
+      <c r="O63" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/mrclaysspeechins00clay/mrclaysspeechins00clay</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
@@ -4929,7 +5017,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O64" s="2" t="n"/>
+      <c r="O64" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/first-annual-message-2</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
@@ -5205,7 +5297,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O68" s="2" t="n"/>
+      <c r="O68" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/veto-message-471</t>
+        </is>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
@@ -5615,7 +5711,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O74" s="2" t="n"/>
+      <c r="O74" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/library/document/fort-hill-address/</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
@@ -5753,7 +5853,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O76" s="2" t="n"/>
+      <c r="O76" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/speech-on-the-presidential-veto-of-the-bank-bill-sop/</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
@@ -5891,7 +5995,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O78" s="2" t="n"/>
+      <c r="O78" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/19th_century/jack01.asp</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
@@ -6849,7 +6957,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O92" s="2" t="n"/>
+      <c r="O92" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/appeal-of-the-independent-democrats-in-congress-to-the-american-people/</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="n">
@@ -6920,7 +7032,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O93" s="2" t="n"/>
+      <c r="O93" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/nebraska-territory/</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="2" t="n">
@@ -7133,7 +7249,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O96" s="2" t="n"/>
+      <c r="O96" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/lincoln-douglas-debates/</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="n">
@@ -7204,7 +7324,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O97" s="2" t="n"/>
+      <c r="O97" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/19th_century/csa_scarsec.asp</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="2" t="n">
@@ -7275,7 +7399,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O98" s="2" t="n"/>
+      <c r="O98" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/19th_century/lincoln1.asp</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="n">
@@ -7346,7 +7474,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O99" s="2" t="n"/>
+      <c r="O99" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/19th_century/csa_m042961.asp</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="n">
@@ -7417,7 +7549,11 @@
           <t>partial in volume</t>
         </is>
       </c>
-      <c r="O100" s="2" t="n"/>
+      <c r="O100" s="2" t="inlineStr">
+        <is>
+          <t>https://housedivided.dickinson.edu/sites/lincoln/letter-to-horace-greeley-august-22-1862/</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="n">
@@ -7488,7 +7624,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O101" s="2" t="n"/>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>https://www.archives.gov/exhibits/featured-documents/emancipation-proclamation/transcript.html</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="n">
@@ -7630,7 +7770,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O103" s="2" t="n"/>
+      <c r="O103" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/proclamation-115-concerning-bill-guarantee-certain-states-whose-governments-have-been</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="n">
@@ -7701,7 +7845,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O104" s="2" t="n"/>
+      <c r="O104" s="2" t="inlineStr">
+        <is>
+          <t>https://hd.housedivided.dickinson.edu/node/42761</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="n">
@@ -7839,7 +7987,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O106" s="2" t="n"/>
+      <c r="O106" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nps.gov/linc/learn/historyculture/lincoln-second-inaugural.htm</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="n">
@@ -7910,7 +8062,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O107" s="2" t="n"/>
+      <c r="O107" s="2" t="inlineStr">
+        <is>
+          <t>https://housedivided.dickinson.edu/sites/lincoln/last-speech-april-11-1865/</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="n">
@@ -7981,7 +8137,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O108" s="2" t="n"/>
+      <c r="O108" s="2" t="inlineStr">
+        <is>
+          <t>https://web.mit.edu/21h.102/www/Primary%20source%20collections/Reconstruction/Stevens,%20Speech%20on%20reconstruction.html</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="n">
@@ -8959,7 +9119,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O122" s="2" t="n"/>
+      <c r="O122" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/ebooks/55308</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="n">
@@ -9373,7 +9537,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O128" s="2" t="n"/>
+      <c r="O128" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/ebooks/624</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="n">
@@ -9440,7 +9608,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O129" s="2" t="n"/>
+      <c r="O129" s="2" t="inlineStr">
+        <is>
+          <t>https://media.carnegie.org/filer_public/ab/c9/abc9fb4b-dc86-4ce8-ae31-a983b9a326ed/ccny_essay_1889_thegospelofwealth.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="n">
@@ -9574,7 +9746,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O131" s="2" t="n"/>
+      <c r="O131" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/populist-party-platform-1892</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="n">
@@ -9712,7 +9888,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O133" s="2" t="n"/>
+      <c r="O133" s="2" t="inlineStr">
+        <is>
+          <t>https://millercenter.org/the-presidency/presidential-speeches/august-8-1893-special-session-message</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="n">
@@ -9783,7 +9963,11 @@
           <t>partial in volume</t>
         </is>
       </c>
-      <c r="O134" s="2" t="n"/>
+      <c r="O134" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikisource.org/wiki/War_and_Other_Essays/The_Absurd_Effort_to_Make_the_World_Over</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="n">
@@ -9850,7 +10034,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O135" s="2" t="n"/>
+      <c r="O135" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/files/60473/60473-h/60473-h.htm</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="n">
@@ -9988,7 +10176,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O137" s="2" t="n"/>
+      <c r="O137" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/coinsfinancialsc00harvrich</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="n">
@@ -10927,7 +11119,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O150" s="2" t="n"/>
+      <c r="O150" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/message-congress-requesting-declaration-war-with-spain</t>
+        </is>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="n">
@@ -10994,7 +11190,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O151" s="2" t="n"/>
+      <c r="O151" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/platform-of-american-anti-imperialist-league/</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="n">
@@ -11124,7 +11324,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O153" s="2" t="n"/>
+      <c r="O153" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/ebooks/54710</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="n">
@@ -11191,7 +11395,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O154" s="2" t="n"/>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/ebooks/2810</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="n">
@@ -11692,7 +11900,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O161" s="2" t="n"/>
+      <c r="O161" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/oldorderchangeth00whit</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="n">
@@ -11893,7 +12105,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O164" s="2" t="n"/>
+      <c r="O164" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/ebooks/14811</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="n">
@@ -11960,7 +12176,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O165" s="2" t="n"/>
+      <c r="O165" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/ebooks/10485</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="n">
@@ -12098,7 +12318,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O167" s="2" t="n"/>
+      <c r="O167" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/wilson1.asp</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="n">
@@ -12165,7 +12389,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O168" s="2" t="n"/>
+      <c r="O168" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/cache/epub/79553/pg79553-images.html</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" s="2" t="n">
@@ -12236,7 +12464,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O169" s="2" t="n"/>
+      <c r="O169" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/message-neutrality</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="n">
@@ -12374,7 +12606,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O171" s="2" t="n"/>
+      <c r="O171" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-the-senate-the-united-states-world-league-for-peace</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="n">
@@ -12445,7 +12681,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O172" s="2" t="n"/>
+      <c r="O172" s="2" t="inlineStr">
+        <is>
+          <t>https://www.archives.gov/milestone-documents/address-to-congress-declaration-of-war-against-germany</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="n">
@@ -12516,7 +12756,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O173" s="2" t="n"/>
+      <c r="O173" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/opposition-to-war/</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="n">
@@ -12587,7 +12831,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O174" s="2" t="n"/>
+      <c r="O174" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/wilson14.asp</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="n">
@@ -12804,7 +13052,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O177" s="2" t="n"/>
+      <c r="O177" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-the-third-plenary-session-the-peace-conference-paris-france</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="n">
@@ -13088,7 +13340,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O181" s="2" t="n"/>
+      <c r="O181" s="2" t="inlineStr">
+        <is>
+          <t>https://www.senate.gov/artandhistory/history/common/generic/Speeches_Borah_League.htm</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="n">
@@ -13222,7 +13478,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O183" s="2" t="n"/>
+      <c r="O183" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/progressive-party-platform-1924</t>
+        </is>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="n">
@@ -13427,7 +13687,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O186" s="2" t="n"/>
+      <c r="O186" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/campaign-address-new-york-city</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="n">
@@ -13565,7 +13829,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O188" s="2" t="n"/>
+      <c r="O188" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/campaign-address-progressive-government-the-commonwealth-club-san-francisco-california</t>
+        </is>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="n">
@@ -13636,7 +13904,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O189" s="2" t="n"/>
+      <c r="O189" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/froos1.asp</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="n">
@@ -13995,7 +14267,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O194" s="2" t="n"/>
+      <c r="O194" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/fireside-chat-17</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="n">
@@ -14137,7 +14413,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O196" s="2" t="n"/>
+      <c r="O196" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-chicago</t>
+        </is>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="n">
@@ -14208,7 +14488,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O197" s="2" t="n"/>
+      <c r="O197" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/press-conference-3</t>
+        </is>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="n">
@@ -14279,7 +14563,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O198" s="2" t="n"/>
+      <c r="O198" s="2" t="inlineStr">
+        <is>
+          <t>https://www.archives.gov/milestone-documents/president-franklin-roosevelts-annual-message-to-congress</t>
+        </is>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="n">
@@ -14421,7 +14709,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O200" s="2" t="n"/>
+      <c r="O200" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/america-first/</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="n">
@@ -14555,7 +14847,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O202" s="2" t="n"/>
+      <c r="O202" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/wwii/atlantic.asp</t>
+        </is>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="n">
@@ -14626,7 +14922,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O203" s="2" t="n"/>
+      <c r="O203" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-congress-requesting-declaration-war-with-japan</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="n">
@@ -14752,7 +15052,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O205" s="2" t="n"/>
+      <c r="O205" s="2" t="inlineStr">
+        <is>
+          <t>https://www.trumanlibrary.gov/library/public-papers/93/statement-president-announcing-use-bomb-hiroshima</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="n">
@@ -14957,7 +15261,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O208" s="2" t="n"/>
+      <c r="O208" s="2" t="inlineStr">
+        <is>
+          <t>https://www.trumanlibrary.gov/library/public-papers/56/special-message-congress-greece-and-turkey-truman-doctrine</t>
+        </is>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="n">
@@ -15028,7 +15336,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O209" s="2" t="n"/>
+      <c r="O209" s="2" t="inlineStr">
+        <is>
+          <t>https://www.marshallfoundation.org/the-marshall-plan/speech/</t>
+        </is>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="n">
@@ -15233,7 +15545,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O212" s="2" t="n"/>
+      <c r="O212" s="2" t="inlineStr">
+        <is>
+          <t>https://irp.fas.org/offdocs/nsc-hst/nsc-68.htm</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="n">
@@ -15304,7 +15620,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O213" s="2" t="n"/>
+      <c r="O213" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/app/details/SERIALSET-11511_00_00-019-0036-0000</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" s="2" t="n">
@@ -15509,7 +15829,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O216" s="2" t="n"/>
+      <c r="O216" s="2" t="inlineStr">
+        <is>
+          <t>https://docsteach.org/document/korean-armistice-agreement/</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="n">
@@ -15860,7 +16184,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O221" s="2" t="n"/>
+      <c r="O221" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/southern-manifesto/</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" s="2" t="n">
@@ -16002,7 +16330,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O223" s="2" t="n"/>
+      <c r="O223" s="2" t="inlineStr">
+        <is>
+          <t>https://www.archives.gov/milestone-documents/president-dwight-d-eisenhowers-farewell-address</t>
+        </is>
+      </c>
     </row>
     <row r="224">
       <c r="A224" s="2" t="n">
@@ -16073,7 +16405,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O224" s="2" t="n"/>
+      <c r="O224" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/inaugural-address-2</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" s="2" t="n">
@@ -16211,7 +16547,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O226" s="2" t="n"/>
+      <c r="O226" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/commencement-address-yale-university</t>
+        </is>
+      </c>
     </row>
     <row r="227">
       <c r="A227" s="2" t="n">
@@ -16412,7 +16752,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O229" s="2" t="n"/>
+      <c r="O229" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/radio-and-television-report-the-american-people-the-soviet-arms-buildup-cuba</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="2" t="n">
@@ -16684,7 +17028,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O233" s="2" t="n"/>
+      <c r="O233" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/radio-and-television-address-the-american-people-the-nuclear-test-ban-treaty</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" s="2" t="n">
@@ -16889,7 +17237,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O236" s="2" t="n"/>
+      <c r="O236" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/special-message-the-congress-proposing-nationwide-war-the-sources-poverty</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" s="2" t="n">
@@ -17177,7 +17529,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O240" s="2" t="n"/>
+      <c r="O240" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/special-message-the-congress-the-american-promise</t>
+        </is>
+      </c>
     </row>
     <row r="241">
       <c r="A241" s="2" t="n">
@@ -17248,7 +17604,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O241" s="2" t="n"/>
+      <c r="O241" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-johns-hopkins-university-peace-without-conquest</t>
+        </is>
+      </c>
     </row>
     <row r="242">
       <c r="A242" s="2" t="n">
@@ -17319,7 +17679,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O242" s="2" t="n"/>
+      <c r="O242" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lbjlibrary.org/object/text/commencement-address-howard-university-fulfill-these-rights-06-04-1965</t>
+        </is>
+      </c>
     </row>
     <row r="243">
       <c r="A243" s="2" t="n">
@@ -17382,7 +17746,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O243" s="2" t="n"/>
+      <c r="O243" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-the-signing-the-immigration-bill-liberty-island-new-york</t>
+        </is>
+      </c>
     </row>
     <row r="244">
       <c r="A244" s="2" t="n">
@@ -17855,7 +18223,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O250" s="2" t="n"/>
+      <c r="O250" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/annual-message-the-congress-the-economic-report-the-president-12</t>
+        </is>
+      </c>
     </row>
     <row r="251">
       <c r="A251" s="2" t="n">
@@ -17926,7 +18298,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O251" s="2" t="n"/>
+      <c r="O251" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/inaugural-address-1</t>
+        </is>
+      </c>
     </row>
     <row r="252">
       <c r="A252" s="2" t="n">
@@ -18399,7 +18775,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O258" s="2" t="n"/>
+      <c r="O258" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/statement-about-desegregation-elementary-and-secondary-schools</t>
+        </is>
+      </c>
     </row>
     <row r="259">
       <c r="A259" s="4" t="n">
@@ -18738,7 +19118,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O263" s="2" t="n"/>
+      <c r="O263" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-the-nation-outlining-new-economic-policy-the-challenge-peace</t>
+        </is>
+      </c>
     </row>
     <row r="264">
       <c r="A264" s="4" t="n">
@@ -18801,7 +19185,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O264" s="2" t="n"/>
+      <c r="O264" s="2" t="inlineStr">
+        <is>
+          <t>https://scholarlycommons.law.wlu.edu/powellmemo/1</t>
+        </is>
+      </c>
     </row>
     <row r="265">
       <c r="A265" s="4" t="n">
@@ -18931,7 +19319,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O266" s="2" t="n"/>
+      <c r="O266" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/veto-the-economic-opportunity-amendments-1971</t>
+        </is>
+      </c>
     </row>
     <row r="267">
       <c r="A267" s="4" t="n">
@@ -19207,7 +19599,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O270" s="2" t="n"/>
+      <c r="O270" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-joint-session-the-congress-return-from-austria-the-soviet-union-iran-and-poland</t>
+        </is>
+      </c>
     </row>
     <row r="271">
       <c r="A271" s="4" t="n">
@@ -19349,7 +19745,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O272" s="2" t="n"/>
+      <c r="O272" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-signing-proclamation-granting-pardon-richard-nixon</t>
+        </is>
+      </c>
     </row>
     <row r="273">
       <c r="A273" s="4" t="n">
@@ -19814,7 +20214,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O279" s="2" t="n"/>
+      <c r="O279" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-before-joint-session-the-congress-the-camp-david-meeting-the-middle-east</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" s="4" t="n">
@@ -20015,7 +20419,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O282" s="2" t="n"/>
+      <c r="O282" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-the-nation-energy-and-national-goals-the-malaise-speech</t>
+        </is>
+      </c>
     </row>
     <row r="283">
       <c r="A283" s="4" t="n">
@@ -20086,7 +20494,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O283" s="2" t="n"/>
+      <c r="O283" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/rescue-attempt-for-american-hostages-iran-letter-the-speaker-the-house-and-the-president</t>
+        </is>
+      </c>
     </row>
     <row r="284">
       <c r="A284" s="4" t="n">
@@ -20303,7 +20715,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O286" s="2" t="n"/>
+      <c r="O286" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/presidential-debate-cleveland</t>
+        </is>
+      </c>
     </row>
     <row r="287">
       <c r="A287" s="4" t="n">
@@ -20425,7 +20841,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O288" s="2" t="n"/>
+      <c r="O288" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/inaugural-address-11</t>
+        </is>
+      </c>
     </row>
     <row r="289">
       <c r="A289" s="4" t="n">
@@ -20488,7 +20908,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O289" s="2" t="n"/>
+      <c r="O289" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-and-question-and-answer-session-with-reporters-the-air-traffic-controllers-strike</t>
+        </is>
+      </c>
     </row>
     <row r="290">
       <c r="A290" s="4" t="n">
@@ -20622,7 +21046,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O291" s="2" t="n"/>
+      <c r="O291" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-members-the-national-press-club-arms-reduction-and-nuclear-weapons</t>
+        </is>
+      </c>
     </row>
     <row r="292">
       <c r="A292" s="4" t="n">
@@ -20815,7 +21243,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O294" s="2" t="n"/>
+      <c r="O294" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reaganlibrary.gov/archives/speech/remarks-annual-convention-national-association-evangelicals-orlando-fl</t>
+        </is>
+      </c>
     </row>
     <row r="295">
       <c r="A295" s="4" t="n">
@@ -20878,7 +21310,11 @@
           <t>month only</t>
         </is>
       </c>
-      <c r="O295" s="2" t="n"/>
+      <c r="O295" s="2" t="inlineStr">
+        <is>
+          <t>https://eric.ed.gov/?id=ED226006</t>
+        </is>
+      </c>
     </row>
     <row r="296">
       <c r="A296" s="4" t="n">
@@ -21075,7 +21511,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O298" s="2" t="n"/>
+      <c r="O298" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/statement-signing-the-immigration-reform-and-control-act-1986</t>
+        </is>
+      </c>
     </row>
     <row r="299">
       <c r="A299" s="4" t="n">
@@ -21516,7 +21956,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O305" s="2" t="n"/>
+      <c r="O305" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-signing-the-americans-with-disabilities-act-1990</t>
+        </is>
+      </c>
     </row>
     <row r="306">
       <c r="A306" s="4" t="n">
@@ -21977,7 +22421,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O312" s="2" t="n"/>
+      <c r="O312" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-signing-the-north-american-free-trade-agreement-implementation-act</t>
+        </is>
+      </c>
     </row>
     <row r="313">
       <c r="A313" s="4" t="n">
@@ -22300,7 +22748,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O317" s="2" t="n"/>
+      <c r="O317" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-before-joint-session-the-congress-the-state-the-union-10</t>
+        </is>
+      </c>
     </row>
     <row r="318">
       <c r="A318" s="4" t="n">
@@ -22832,7 +23284,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O325" s="2" t="n"/>
+      <c r="O325" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-signing-legislation-permanent-normal-trade-relations-with-china</t>
+        </is>
+      </c>
     </row>
     <row r="326">
       <c r="A326" s="4" t="n">
@@ -23029,7 +23485,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O328" s="2" t="n"/>
+      <c r="O328" s="2" t="inlineStr">
+        <is>
+          <t>https://georgewbush-whitehouse.archives.gov/news/releases/2001/09/20010920-8.html</t>
+        </is>
+      </c>
     </row>
     <row r="329">
       <c r="A329" s="4" t="n">
@@ -23226,7 +23686,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O331" s="2" t="n"/>
+      <c r="O331" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/address-before-joint-session-the-congress-the-state-the-union-22</t>
+        </is>
+      </c>
     </row>
     <row r="332">
       <c r="A332" s="4" t="n">
@@ -23419,7 +23883,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O334" s="2" t="n"/>
+      <c r="O334" s="2" t="inlineStr">
+        <is>
+          <t>https://georgewbush-whitehouse.archives.gov/news/releases/2003/02/20030205-1.html</t>
+        </is>
+      </c>
     </row>
     <row r="335">
       <c r="A335" s="4" t="n">
@@ -25511,7 +25979,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O366" s="2" t="n"/>
+      <c r="O366" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/inaugural-address-14</t>
+        </is>
+      </c>
     </row>
     <row r="367">
       <c r="A367" s="2" t="n">
@@ -25834,7 +26306,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O371" s="2" t="n"/>
+      <c r="O371" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/joint-statement-president-trump-and-chairman-the-state-affairs-commission-kim-jong-un</t>
+        </is>
+      </c>
     </row>
     <row r="372">
       <c r="A372" s="2" t="n">
@@ -26488,7 +26964,11 @@
           <t>month only</t>
         </is>
       </c>
-      <c r="O381" s="2" t="n"/>
+      <c r="O381" s="2" t="inlineStr">
+        <is>
+          <t>https://static.heritage.org/project2025/2025_MandateForLeadership_FULL.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="382">
       <c r="A382" s="2" t="n">

</xml_diff>

<commit_message>
T-0065: add reviewed probable links; Gutenberg links point at the read-online page
41 links the editor spot-checked, minus the ones I know point at the wrong document or
cannot be opened. No unz.com links.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Object_Matrix.xlsx
+++ b/editorial/NTK_Backstory_Object_Matrix.xlsx
@@ -1193,7 +1193,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O10" s="2" t="n"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/cache/epub/47111/pg47111-images.html</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
@@ -1473,7 +1477,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O14" s="2" t="n"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/cache/epub/45205/pg45205-images.html</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
@@ -1544,7 +1552,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O15" s="2" t="n"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/cache/epub/45205/pg45205-images.html</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
@@ -1615,7 +1627,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O16" s="2" t="n"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/cache/epub/5655/pg5655-images.html</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
@@ -2124,7 +2140,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O23" s="2" t="n"/>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>https://www.econlib.org/library/Smith/smWN.html?chapter_num=37#book-reader</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
@@ -2534,7 +2554,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O29" s="2" t="n"/>
+      <c r="O29" s="2" t="inlineStr">
+        <is>
+          <t>https://www.lva.virginia.gov/collections/educator-resources/dbva/files/original/3538b34674838abbb424ba9ef79caabb.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
@@ -2605,7 +2629,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O30" s="2" t="n"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>https://www.loc.gov/resource/mgw2.013/?sp=139</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
@@ -2889,7 +2917,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O34" s="2" t="n"/>
+      <c r="O34" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/fed10.asp</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="n">
@@ -2960,7 +2992,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O35" s="2" t="n"/>
+      <c r="O35" s="2" t="inlineStr">
+        <is>
+          <t>https://founders.archives.gov/documents/Jefferson/01-12-02-0454</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="2" t="n">
@@ -3027,7 +3063,11 @@
           <t>partial in volume</t>
         </is>
       </c>
-      <c r="O36" s="2" t="n"/>
+      <c r="O36" s="2" t="inlineStr">
+        <is>
+          <t>https://www.loc.gov/resource/law.lled003/?st=gallery</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
@@ -3098,7 +3138,11 @@
           <t>partial in volume</t>
         </is>
       </c>
-      <c r="O37" s="2" t="n"/>
+      <c r="O37" s="2" t="inlineStr">
+        <is>
+          <t>https://founders.archives.gov/documents/Hamilton/01-06-02-0076-0002-0001</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="n">
@@ -3524,7 +3568,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O43" s="2" t="n"/>
+      <c r="O43" s="2" t="inlineStr">
+        <is>
+          <t>https://founders.archives.gov/documents/Hamilton/01-10-02-0001-0007</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
@@ -3591,7 +3639,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O44" s="2" t="n"/>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>https://babel.hathitrust.org/cgi/pt?id=mdp.35112204851705</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
@@ -3658,7 +3710,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O45" s="2" t="n"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>https://founders.archives.gov/documents/Hamilton/01-18-02-0305-0002</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
@@ -4017,7 +4073,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O50" s="2" t="n"/>
+      <c r="O50" s="2" t="inlineStr">
+        <is>
+          <t>https://founders.archives.gov/documents/Jefferson/01-37-02-0220</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
@@ -4508,7 +4568,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O57" s="2" t="n"/>
+      <c r="O57" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/19th_century/hartconv.asp</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
@@ -4721,7 +4785,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O60" s="2" t="n"/>
+      <c r="O60" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/reportsofproceed00newy</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
@@ -5092,7 +5160,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O65" s="2" t="n"/>
+      <c r="O65" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikisource.org/wiki/South_Carolina_Exposition_and_Protest</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
@@ -7699,7 +7771,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O102" s="2" t="n"/>
+      <c r="O102" s="2" t="inlineStr">
+        <is>
+          <t>https://www.loc.gov/item/mal4356500/</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="n">
@@ -7916,7 +7992,11 @@
           <t>partial in volume</t>
         </is>
       </c>
-      <c r="O105" s="2" t="n"/>
+      <c r="O105" s="2" t="inlineStr">
+        <is>
+          <t>http://people.sunyulster.edu/voughth/Alexandria_Petition.htm</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="n">
@@ -8208,7 +8288,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O109" s="2" t="n"/>
+      <c r="O109" s="2" t="inlineStr">
+        <is>
+          <t>https://ldhi.library.cofc.edu/exhibits/show/after_slavery_educator/unit_five_documents/document_five</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="2" t="n">
@@ -8417,7 +8501,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O112" s="2" t="n"/>
+      <c r="O112" s="2" t="inlineStr">
+        <is>
+          <t>https://www.famous-trials.com/johnson/478-sumneropinion</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="n">
@@ -8484,7 +8572,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O113" s="2" t="n"/>
+      <c r="O113" s="2" t="inlineStr">
+        <is>
+          <t>https://www.famous-trials.com/johnson/476-grimesopinion</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="n">
@@ -8902,7 +8994,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O119" s="2" t="n"/>
+      <c r="O119" s="2" t="inlineStr">
+        <is>
+          <t>https://collections.americanantiquarian.org/blackpublishing/items/show/10751</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="n">
@@ -9121,7 +9217,7 @@
       </c>
       <c r="O122" s="2" t="inlineStr">
         <is>
-          <t>https://www.gutenberg.org/ebooks/55308</t>
+          <t>https://www.gutenberg.org/cache/epub/55308/pg55308-images.html</t>
         </is>
       </c>
     </row>
@@ -9470,7 +9566,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O127" s="2" t="n"/>
+      <c r="O127" s="2" t="inlineStr">
+        <is>
+          <t>https://www.loc.gov/item/33039235/</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="n">
@@ -9539,7 +9639,7 @@
       </c>
       <c r="O128" s="2" t="inlineStr">
         <is>
-          <t>https://www.gutenberg.org/ebooks/624</t>
+          <t>https://www.gutenberg.org/cache/epub/624/pg624-images.html</t>
         </is>
       </c>
     </row>
@@ -11326,7 +11426,7 @@
       </c>
       <c r="O153" s="2" t="inlineStr">
         <is>
-          <t>https://www.gutenberg.org/ebooks/54710</t>
+          <t>https://www.gutenberg.org/cache/epub/54710/pg54710-images.html</t>
         </is>
       </c>
     </row>
@@ -11397,7 +11497,7 @@
       </c>
       <c r="O154" s="2" t="inlineStr">
         <is>
-          <t>https://www.gutenberg.org/ebooks/2810</t>
+          <t>https://www.gutenberg.org/cache/epub/2810/pg2810-images.html</t>
         </is>
       </c>
     </row>
@@ -12107,7 +12207,7 @@
       </c>
       <c r="O164" s="2" t="inlineStr">
         <is>
-          <t>https://www.gutenberg.org/ebooks/14811</t>
+          <t>https://www.gutenberg.org/cache/epub/14811/pg14811-images.html</t>
         </is>
       </c>
     </row>
@@ -12178,7 +12278,7 @@
       </c>
       <c r="O165" s="2" t="inlineStr">
         <is>
-          <t>https://www.gutenberg.org/ebooks/10485</t>
+          <t>https://www.gutenberg.org/cache/epub/10485/pg10485-images.html</t>
         </is>
       </c>
     </row>
@@ -13616,7 +13716,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O185" s="2" t="n"/>
+      <c r="O185" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/Klansfightamericanism</t>
+        </is>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="n">
@@ -15190,7 +15294,11 @@
           <t>partial in volume</t>
         </is>
       </c>
-      <c r="O207" s="2" t="n"/>
+      <c r="O207" s="2" t="inlineStr">
+        <is>
+          <t>https://www.foreignaffairs.com/articles/russian-federation/1947-07-01/sources-soviet-conduct</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="n">
@@ -16050,7 +16158,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O219" s="2" t="n"/>
+      <c r="O219" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/the-presidents-news-conference-453</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="n">
@@ -17095,7 +17207,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O234" s="2" t="n"/>
+      <c r="O234" s="2" t="inlineStr">
+        <is>
+          <t>https://treaties.unoda.org/t/test_ban/text</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" s="2" t="n">
@@ -17166,7 +17282,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O235" s="2" t="n"/>
+      <c r="O235" s="2" t="inlineStr">
+        <is>
+          <t>https://www.loc.gov/static/programs/national-recording-preservation-board/documents/IHaveADream.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="236">
       <c r="A236" s="2" t="n">
@@ -17817,7 +17937,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O244" s="2" t="n"/>
+      <c r="O244" s="2" t="inlineStr">
+        <is>
+          <t>https://web.viu.ca/davies/H323Vietnam/Fulbright.ArroganceofPower.1966.htm</t>
+        </is>
+      </c>
     </row>
     <row r="245">
       <c r="A245" s="2" t="n">
@@ -17955,7 +18079,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O246" s="2" t="n"/>
+      <c r="O246" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ojp.gov/ncjrs/virtual-library/abstracts/national-advisory-commission-civil-disorders-report</t>
+        </is>
+      </c>
     </row>
     <row r="247">
       <c r="A247" s="2" t="n">
@@ -18633,7 +18761,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O256" s="2" t="n"/>
+      <c r="O256" s="2" t="inlineStr">
+        <is>
+          <t>https://www.nixonlibrary.gov/sites/default/files/virtuallibrary/documents/jul10/53.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="257">
       <c r="A257" s="4" t="n">
@@ -19461,7 +19593,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O268" s="2" t="n"/>
+      <c r="O268" s="2" t="inlineStr">
+        <is>
+          <t>http://www.taiwandocuments.org/communique01.htm</t>
+        </is>
+      </c>
     </row>
     <row r="269">
       <c r="A269" s="4" t="n">
@@ -20975,7 +21111,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O290" s="2" t="n"/>
+      <c r="O290" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-signing-the-economic-recovery-tax-act-1981-and-the-omnibus-budget-reconciliation</t>
+        </is>
+      </c>
     </row>
     <row r="291">
       <c r="A291" s="4" t="n">
@@ -21763,7 +21903,11 @@
           <t>year only</t>
         </is>
       </c>
-      <c r="O302" s="2" t="n"/>
+      <c r="O302" s="2" t="inlineStr">
+        <is>
+          <t>https://pages.ucsd.edu/~bslantchev/courses/pdf/Fukuyama%20-%20End%20of%20History.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="303">
       <c r="A303" s="4" t="n">
@@ -22555,7 +22699,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O314" s="2" t="n"/>
+      <c r="O314" s="2" t="inlineStr">
+        <is>
+          <t>https://billofrightsinstitute.org/activities/republican-house-representatives-republican-contract-with-america-1994</t>
+        </is>
+      </c>
     </row>
     <row r="315">
       <c r="A315" s="4" t="n">
@@ -23753,7 +23901,11 @@
           <t>month only</t>
         </is>
       </c>
-      <c r="O332" s="2" t="n"/>
+      <c r="O332" s="2" t="inlineStr">
+        <is>
+          <t>https://georgewbush-whitehouse.archives.gov/nsc/nss/2002/</t>
+        </is>
+      </c>
     </row>
     <row r="333">
       <c r="A333" s="4" t="n">
@@ -25065,7 +25217,11 @@
           <t>month only</t>
         </is>
       </c>
-      <c r="O352" s="2" t="n"/>
+      <c r="O352" s="2" t="inlineStr">
+        <is>
+          <t>https://wearethe99percent.tumblr.com/</t>
+        </is>
+      </c>
     </row>
     <row r="353">
       <c r="A353" s="2" t="n">
@@ -26176,7 +26332,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O369" s="2" t="n"/>
+      <c r="O369" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/DTIC_AD1046463</t>
+        </is>
+      </c>
     </row>
     <row r="370">
       <c r="A370" s="2" t="n">
@@ -26440,7 +26600,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O373" s="2" t="n"/>
+      <c r="O373" s="2" t="inlineStr">
+        <is>
+          <t>https://www.businessroundtable.org/business-roundtable-redefines-the-purpose-of-a-corporation-to-promote-an-economy-that-serves-all-americans</t>
+        </is>
+      </c>
     </row>
     <row r="374">
       <c r="A374" s="2" t="n">

</xml_diff>

<commit_message>
T-0065: link 20 more objects (second research pass)
Verified links only; 16 probable are in the review sheet.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Object_Matrix.xlsx
+++ b/editorial/NTK_Backstory_Object_Matrix.xlsx
@@ -838,7 +838,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O5" s="2" t="n"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/bim_eighteenth-century_the-objections-to-the-ta_jenyns-soame_1765</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
@@ -905,7 +909,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O6" s="2" t="n"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/bim_eighteenth-century_considerations-on-the-pr_dulany-daniel_1765</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
@@ -4223,7 +4231,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O52" s="2" t="n"/>
+      <c r="O52" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/letters-protesting-the-louisiana-purchase/</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
@@ -6619,7 +6631,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O86" s="2" t="n"/>
+      <c r="O86" s="2" t="inlineStr">
+        <is>
+          <t>https://millercenter.org/the-presidency/presidential-speeches/may-11-1846-war-message-congress</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="n">
@@ -6895,7 +6911,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O90" s="2" t="n"/>
+      <c r="O90" s="2" t="inlineStr">
+        <is>
+          <t>https://www.gutenberg.org/cache/epub/203/pg203-images.html</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="2" t="n">
@@ -11858,7 +11878,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O159" s="2" t="n"/>
+      <c r="O159" s="2" t="inlineStr">
+        <is>
+          <t>https://www.congress.gov/59/crecb/1906/02/07/GPO-CRECB-1906-pt3-v40-4-2.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="n">
@@ -12138,7 +12162,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O163" s="2" t="n"/>
+      <c r="O163" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/my-confession-of-faith-speech-before-the-progressive-party-national-convention/</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="n">
@@ -14300,7 +14328,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O193" s="2" t="n"/>
+      <c r="O193" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/this-challenge-to-liberty/</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="n">
@@ -14446,7 +14478,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O195" s="2" t="n"/>
+      <c r="O195" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/app/details/SERIALSET-10076_00_00-356-0711-0000</t>
+        </is>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="n">
@@ -15874,7 +15910,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O215" s="2" t="n"/>
+      <c r="O215" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/statement-on-liberation-policy/</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="n">
@@ -18213,7 +18253,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O248" s="2" t="n"/>
+      <c r="O248" s="2" t="inlineStr">
+        <is>
+          <t>https://www.un.org/en/conf/npt/2005/npttreaty.html</t>
+        </is>
+      </c>
     </row>
     <row r="249">
       <c r="A249" s="2" t="n">
@@ -18690,7 +18734,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O255" s="2" t="n"/>
+      <c r="O255" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/statement-about-the-national-environmental-policy-act-1969</t>
+        </is>
+      </c>
     </row>
     <row r="256">
       <c r="A256" s="4" t="n">
@@ -22167,7 +22215,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O306" s="2" t="n"/>
+      <c r="O306" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/statement-signing-the-bill-amending-the-clean-air-act</t>
+        </is>
+      </c>
     </row>
     <row r="307">
       <c r="A307" s="4" t="n">
@@ -22766,7 +22818,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O315" s="2" t="n"/>
+      <c r="O315" s="2" t="inlineStr">
+        <is>
+          <t>https://peacemaker.un.org/en/node/9207</t>
+        </is>
+      </c>
     </row>
     <row r="316">
       <c r="A316" s="4" t="n">
@@ -24236,7 +24292,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O337" s="2" t="n"/>
+      <c r="O337" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/features/911-commission-report</t>
+        </is>
+      </c>
     </row>
     <row r="338">
       <c r="A338" s="4" t="n">
@@ -24299,7 +24359,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O338" s="2" t="n"/>
+      <c r="O338" s="2" t="inlineStr">
+        <is>
+          <t>https://md.china-embassy.gov.cn/eng/zgjj/200503/t20050314_2732280.htm</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" s="4" t="n">
@@ -24823,7 +24887,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O346" s="2" t="n"/>
+      <c r="O346" s="2" t="inlineStr">
+        <is>
+          <t>https://www.presidency.ucsb.edu/documents/remarks-cairo</t>
+        </is>
+      </c>
     </row>
     <row r="347">
       <c r="A347" s="2" t="n">
@@ -25284,7 +25352,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O353" s="2" t="n"/>
+      <c r="O353" s="2" t="inlineStr">
+        <is>
+          <t>https://www.dhs.gov/xlibrary/assets/s1-exercising-prosecutorial-discretion-individuals-who-came-to-us-as-children.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="354">
       <c r="A354" s="2" t="n">
@@ -25879,7 +25951,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O362" s="2" t="n"/>
+      <c r="O362" s="2" t="inlineStr">
+        <is>
+          <t>https://unfccc.int/files/meetings/paris_nov_2015/application/pdf/paris_agreement_english_.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="363">
       <c r="A363" s="2" t="n">
@@ -26667,7 +26743,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O374" s="2" t="n"/>
+      <c r="O374" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/app/details/GOVPUB-S-PURL-gpo132866</t>
+        </is>
+      </c>
     </row>
     <row r="375">
       <c r="A375" s="2" t="n">

</xml_diff>

<commit_message>
T-0065: graduate 16 editor-reviewed probable links
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Object_Matrix.xlsx
+++ b/editorial/NTK_Backstory_Object_Matrix.xlsx
@@ -771,7 +771,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O4" s="2" t="n"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>https://www.ruhr-uni-bochum.de/gna/Quellensammlung/01/01_resolutionvirginia_1764.htm</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="n">
@@ -1059,7 +1063,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O8" s="2" t="n"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>https://en.wikisource.org/wiki/Speech_against_the_Stamp_Act</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
@@ -4655,7 +4663,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O58" s="2" t="n"/>
+      <c r="O58" s="2" t="inlineStr">
+        <is>
+          <t>https://founders.archives.gov/documents/Jefferson/03-12-02-0343-0002</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
@@ -11026,7 +11038,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O147" s="2" t="n"/>
+      <c r="O147" s="2" t="inlineStr">
+        <is>
+          <t>https://www.loc.gov/resource/gdcmassbookdig.crossofgold00dave/?st=gallery</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="n">
@@ -12375,7 +12391,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O166" s="2" t="n"/>
+      <c r="O166" s="2" t="inlineStr">
+        <is>
+          <t>https://catalog.hathitrust.org/Record/001738949</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="n">
@@ -15129,7 +15149,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O204" s="2" t="n"/>
+      <c r="O204" s="2" t="inlineStr">
+        <is>
+          <t>https://www.govinfo.gov/content/pkg/STATUTE-57/pdf/STATUTE-57-Pg1152.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="n">
@@ -15626,7 +15650,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O211" s="2" t="n"/>
+      <c r="O211" s="2" t="inlineStr">
+        <is>
+          <t>https://teachingamericanhistory.org/document/speech-on-the-north-atlantic-treaty/</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="n">
@@ -18671,7 +18699,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O254" s="2" t="n"/>
+      <c r="O254" s="2" t="inlineStr">
+        <is>
+          <t>https://energyhistory.yale.edu/santa-barbara-declaration-of-environmental-rights-1970</t>
+        </is>
+      </c>
     </row>
     <row r="255">
       <c r="A255" s="2" t="n">
@@ -21766,7 +21798,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O299" s="2" t="n"/>
+      <c r="O299" s="2" t="inlineStr">
+        <is>
+          <t>https://digital.library.unt.edu/ark:/67531/metadc1594/m1/48/?q=wtvh</t>
+        </is>
+      </c>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n">
@@ -21829,7 +21865,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O300" s="2" t="n"/>
+      <c r="O300" s="2" t="inlineStr">
+        <is>
+          <t>https://www.reaganlibrary.gov/archives/speech/treaty-between-united-states-america-and-union-soviet-socialist-republics</t>
+        </is>
+      </c>
     </row>
     <row r="301">
       <c r="A301" s="4" t="n">
@@ -21892,7 +21932,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O301" s="2" t="n"/>
+      <c r="O301" s="2" t="inlineStr">
+        <is>
+          <t>https://pulitzercenter.org/sites/default/files/june_23_1988_senate_hearing_1.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="302">
       <c r="A302" s="4" t="n">
@@ -24426,7 +24470,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O339" s="2" t="n"/>
+      <c r="O339" s="2" t="inlineStr">
+        <is>
+          <t>https://2001-2009.state.gov/r/pa/prs/ps/2005/53490.htm</t>
+        </is>
+      </c>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n">
@@ -25088,7 +25136,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O349" s="2" t="n"/>
+      <c r="O349" s="2" t="inlineStr">
+        <is>
+          <t>http://www.state.gov/documents/organization/140035.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="350">
       <c r="A350" s="2" t="n">
@@ -25888,7 +25940,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O361" s="2" t="n"/>
+      <c r="O361" s="2" t="inlineStr">
+        <is>
+          <t>https://2009-2017.state.gov/documents/organization/245317.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="362">
       <c r="A362" s="2" t="n">
@@ -26278,7 +26334,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O367" s="2" t="n"/>
+      <c r="O367" s="2" t="inlineStr">
+        <is>
+          <t>https://trumpwhitehouse.archives.gov/articles/president-trump-announces-u-s-withdrawal-paris-climate-accord/</t>
+        </is>
+      </c>
     </row>
     <row r="368">
       <c r="A368" s="2" t="n">
@@ -26877,7 +26937,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O376" s="2" t="n"/>
+      <c r="O376" s="2" t="inlineStr">
+        <is>
+          <t>https://www.congress.gov/117/crec/2021/01/06/CREC-2021-01-06.pdf</t>
+        </is>
+      </c>
     </row>
     <row r="377">
       <c r="A377" s="2" t="n">

</xml_diff>

<commit_message>
T-0065: graduate 11 editor-supplied links
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Object_Matrix.xlsx
+++ b/editorial/NTK_Backstory_Object_Matrix.xlsx
@@ -1280,7 +1280,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O11" s="2" t="n"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/nationalprivatea00post</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
@@ -3296,7 +3300,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O39" s="2" t="n"/>
+      <c r="O39" s="2" t="inlineStr">
+        <is>
+          <t>https://founders.archives.gov/documents/Hamilton/01-06-02-0234-0002</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
@@ -3876,7 +3884,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O47" s="2" t="n"/>
+      <c r="O47" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/18th_century/virres.asp</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
@@ -6434,7 +6446,11 @@
           <t>not printed</t>
         </is>
       </c>
-      <c r="O83" s="2" t="n"/>
+      <c r="O83" s="2" t="inlineStr">
+        <is>
+          <t>https://docsouth.unc.edu/neh/weld/weld.html</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
@@ -15579,7 +15595,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O210" s="2" t="n"/>
+      <c r="O210" s="2" t="inlineStr">
+        <is>
+          <t>https://avalon.law.yale.edu/20th_century/nato.asp</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="n">
@@ -15867,7 +15887,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O214" s="2" t="n"/>
+      <c r="O214" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/militarysituatio01unit</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="n">
@@ -16439,7 +16463,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O222" s="2" t="n"/>
+      <c r="O222" s="2" t="inlineStr">
+        <is>
+          <t>https://history.state.gov/historicaldocuments/frus1949v09/d22</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" s="2" t="n">
@@ -16861,7 +16889,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O228" s="2" t="n"/>
+      <c r="O228" s="2" t="inlineStr">
+        <is>
+          <t>https://archive.org/details/silentspring00cars</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n">
@@ -19125,7 +19157,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O260" s="2" t="n"/>
+      <c r="O260" s="2" t="inlineStr">
+        <is>
+          <t>https://www.epa.gov/history/epa-history-earth-day</t>
+        </is>
+      </c>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n">
@@ -19890,7 +19926,11 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O271" s="2" t="n"/>
+      <c r="O271" s="2" t="inlineStr">
+        <is>
+          <t>https://watergate.info/impeachment/articles-of-impeachment</t>
+        </is>
+      </c>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n">
@@ -27540,7 +27580,11 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O385" s="2" t="n"/>
+      <c r="O385" s="2" t="inlineStr">
+        <is>
+          <t>https://www.state.gov/new-start/</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:O385"/>

</xml_diff>

<commit_message>
T-0065: pull back 5 links with a specific doubt (lending copy, about-page, hobbyist host, two unopenable pages)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/editorial/NTK_Backstory_Object_Matrix.xlsx
+++ b/editorial/NTK_Backstory_Object_Matrix.xlsx
@@ -16889,11 +16889,7 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O228" s="2" t="inlineStr">
-        <is>
-          <t>https://archive.org/details/silentspring00cars</t>
-        </is>
-      </c>
+      <c r="O228" s="2" t="n"/>
     </row>
     <row r="229">
       <c r="A229" s="2" t="n">
@@ -19157,11 +19153,7 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O260" s="2" t="inlineStr">
-        <is>
-          <t>https://www.epa.gov/history/epa-history-earth-day</t>
-        </is>
-      </c>
+      <c r="O260" s="2" t="n"/>
     </row>
     <row r="261">
       <c r="A261" s="4" t="n">
@@ -19926,11 +19918,7 @@
           <t>from volume</t>
         </is>
       </c>
-      <c r="O271" s="2" t="inlineStr">
-        <is>
-          <t>https://watergate.info/impeachment/articles-of-impeachment</t>
-        </is>
-      </c>
+      <c r="O271" s="2" t="n"/>
     </row>
     <row r="272">
       <c r="A272" s="4" t="n">
@@ -21838,11 +21826,7 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O299" s="2" t="inlineStr">
-        <is>
-          <t>https://digital.library.unt.edu/ark:/67531/metadc1594/m1/48/?q=wtvh</t>
-        </is>
-      </c>
+      <c r="O299" s="2" t="n"/>
     </row>
     <row r="300">
       <c r="A300" s="4" t="n">
@@ -24510,11 +24494,7 @@
           <t>researched</t>
         </is>
       </c>
-      <c r="O339" s="2" t="inlineStr">
-        <is>
-          <t>https://2001-2009.state.gov/r/pa/prs/ps/2005/53490.htm</t>
-        </is>
-      </c>
+      <c r="O339" s="2" t="n"/>
     </row>
     <row r="340">
       <c r="A340" s="4" t="n">

</xml_diff>